<commit_message>
Rebuild Street File as A4 landscape on white paper.
PDF is four landscape pages (black header, crimson rule, amber accents).
xlsx print orientation is landscape on every tab. Dossier photos carry
the stamps so the leverage row stays clear.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sheets/Street-File.xlsx
+++ b/sheets/Street-File.xlsx
@@ -43,18 +43,18 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00C4A35A"/>
+      <color rgb="00FF9F1C"/>
       <sz val="18"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001A1A1A"/>
+      <color rgb="00111111"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="001A1A1A"/>
+      <color rgb="00111111"/>
       <sz val="10"/>
     </font>
     <font>
@@ -66,7 +66,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="009B1B2E"/>
+      <color rgb="00C41E3A"/>
       <sz val="12"/>
     </font>
     <font>
@@ -95,7 +95,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -104,12 +104,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A1A1A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F7F1E6"/>
+        <fgColor rgb="00111111"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,12 +114,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="009B1B2E"/>
+        <fgColor rgb="00C41E3A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF8EC"/>
+        <fgColor rgb="00FFF5E6"/>
       </patternFill>
     </fill>
     <fill>
@@ -134,7 +129,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002C3338"/>
+        <fgColor rgb="001A1A1A"/>
       </patternFill>
     </fill>
   </fills>
@@ -148,23 +143,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B9A989"/>
+        <color rgb="00DDDDDD"/>
       </left>
       <right style="thin">
-        <color rgb="00B9A989"/>
+        <color rgb="00DDDDDD"/>
       </right>
       <top style="thin">
-        <color rgb="00B9A989"/>
+        <color rgb="00DDDDDD"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B9A989"/>
+        <color rgb="00DDDDDD"/>
       </bottom>
     </border>
     <border>
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="00B9A989"/>
+        <color rgb="00DDDDDD"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -172,10 +167,10 @@
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00B9A989"/>
+        <color rgb="00DDDDDD"/>
       </right>
       <top style="thin">
-        <color rgb="00B9A989"/>
+        <color rgb="00DDDDDD"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -184,38 +179,38 @@
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="00B9A989"/>
+        <color rgb="00DDDDDD"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B9A989"/>
+        <color rgb="00DDDDDD"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00B9A989"/>
+        <color rgb="00DDDDDD"/>
       </right>
       <top style="thin">
-        <color rgb="00B9A989"/>
+        <color rgb="00DDDDDD"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B9A989"/>
+        <color rgb="00DDDDDD"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="medium">
-        <color rgb="001A1A1A"/>
+        <color rgb="00111111"/>
       </left>
       <right style="medium">
-        <color rgb="001A1A1A"/>
+        <color rgb="00111111"/>
       </right>
       <top style="medium">
-        <color rgb="001A1A1A"/>
+        <color rgb="00111111"/>
       </top>
       <bottom style="medium">
-        <color rgb="001A1A1A"/>
+        <color rgb="00111111"/>
       </bottom>
     </border>
   </borders>
@@ -231,44 +226,44 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -277,81 +272,81 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -868,7 +863,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="009B1B2E"/>
+    <tabColor rgb="00C41E3A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1169,7 +1164,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;LNC//NET STREET FILE  ·  unofficial table aid&amp;R&amp;A  ·  &amp;P/&amp;N</oddFooter>
@@ -1186,7 +1181,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001A1A1A"/>
+    <tabColor rgb="00111111"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1570,7 +1565,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;LNC//NET STREET FILE  ·  unofficial table aid&amp;R&amp;A  ·  &amp;P/&amp;N</oddFooter>
@@ -1585,7 +1580,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001A1A1A"/>
+    <tabColor rgb="00111111"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2101,7 +2096,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001A1A1A"/>
+    <tabColor rgb="00111111"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2578,7 +2573,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;LNC//NET STREET FILE  ·  unofficial table aid&amp;R&amp;A  ·  &amp;P/&amp;N</oddFooter>
@@ -2593,7 +2588,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="009B1B2E"/>
+    <tabColor rgb="00C41E3A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3266,7 +3261,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00C4A35A"/>
+    <tabColor rgb="00FF9F1C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -4153,7 +4148,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;LNC//NET STREET FILE  ·  unofficial table aid&amp;R&amp;A  ·  &amp;P/&amp;N</oddFooter>
@@ -4682,7 +4677,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;LNC//NET STREET FILE  ·  unofficial table aid&amp;R&amp;A  ·  &amp;P/&amp;N</oddFooter>
@@ -4697,7 +4692,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="009B1B2E"/>
+    <tabColor rgb="00C41E3A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -4917,7 +4912,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;LNC//NET STREET FILE  ·  unofficial table aid&amp;R&amp;A  ·  &amp;P/&amp;N</oddFooter>
@@ -5166,7 +5161,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="002C3338"/>
+    <tabColor rgb="001A1A1A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -5404,7 +5399,7 @@
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;LNC//NET STREET FILE  ·  unofficial table aid&amp;R&amp;A  ·  &amp;P/&amp;N</oddFooter>

</xml_diff>

<commit_message>
Street File: Night Shift PDF/xlsx + DODGE fill
Offline A4 landscape dossier and ledger. PDF filled for Rafael "DODGE" Mora (Lawman 4, H5/Vista); portraits left blank for the player. xlsx has META, Floor 22 ledger, named Backup contacts.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sheets/Street-File.xlsx
+++ b/sheets/Street-File.xlsx
@@ -121,7 +121,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -201,11 +201,80 @@
         <color rgb="00070A0E"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00070A0E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00070A0E"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00070A0E"/>
+      </right>
+      <top style="medium">
+        <color rgb="00070A0E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00070A0E"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00070A0E"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00070A0E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00070A0E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00070A0E"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00070A0E"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -288,6 +357,15 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -377,61 +455,6 @@
     </comment>
   </commentList>
 </comments>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>2</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="838200" cy="838200"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>8</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="838200" cy="838200"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -822,13 +845,6 @@
           <t xml:space="preserve">  STREET FILE   ·   META</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="3" t="n"/>
       <c r="J1" s="3" t="n"/>
       <c r="K1" s="3" t="n"/>
@@ -854,15 +870,23 @@
           <t>Handle</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>DODGE</t>
+        </is>
+      </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Case No.</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="7" t="n"/>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>SF-76-VDR-MORA</t>
+        </is>
+      </c>
+      <c r="E3" s="38" t="n"/>
+      <c r="F3" s="39" t="n"/>
       <c r="G3" s="3" t="n"/>
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
@@ -876,15 +900,19 @@
           <t>Real Name</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Rafael Mora</t>
+        </is>
+      </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="7" t="n"/>
+      <c r="E4" s="38" t="n"/>
+      <c r="F4" s="39" t="n"/>
       <c r="G4" s="3" t="n"/>
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="n"/>
@@ -898,15 +926,19 @@
           <t>Role / Rank</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Lawman 4</t>
+        </is>
+      </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Role 2 / Rank 2</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="7" t="n"/>
+      <c r="E5" s="38" t="n"/>
+      <c r="F5" s="39" t="n"/>
       <c r="G5" s="3" t="n"/>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
@@ -926,9 +958,13 @@
           <t>In-world date</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="7" t="n"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>2076</t>
+        </is>
+      </c>
+      <c r="E6" s="38" t="n"/>
+      <c r="F6" s="39" t="n"/>
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
@@ -954,11 +990,11 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Point buy 62/86 · HUM −2/non-fashion chrome · −4 Borgware (campaign)</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="7" t="n"/>
+          <t>Point buy 62/86 · Neuroport not free (1000eb / HL 7) · company housing free · Backup = named, not dispatch · HUM −2/non-fashion chrome · −4 Borgware (campaign)</t>
+        </is>
+      </c>
+      <c r="E7" s="38" t="n"/>
+      <c r="F7" s="39" t="n"/>
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
@@ -986,11 +1022,6 @@
           <t>RUNNING TOTALS  ·  source of truth (copy Cash / IP / Heat onto PDF page 2 after each session)</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
@@ -1005,7 +1036,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="4" t="inlineStr">
@@ -1013,8 +1044,12 @@
           <t>Trauma Team / subs</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr"/>
-      <c r="F10" s="7" t="n"/>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F10" s="39" t="n"/>
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
@@ -1039,7 +1074,7 @@
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr"/>
-      <c r="F11" s="7" t="n"/>
+      <c r="F11" s="39" t="n"/>
       <c r="G11" s="3" t="n"/>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
@@ -1064,7 +1099,7 @@
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr"/>
-      <c r="F12" s="7" t="n"/>
+      <c r="F12" s="39" t="n"/>
       <c r="G12" s="3" t="n"/>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
@@ -1078,9 +1113,8 @@
           <t>IP earned (all-time)</t>
         </is>
       </c>
-      <c r="B13" s="5">
-        <f>SUM(LEDGER!G4:G43)</f>
-        <v/>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="4" t="inlineStr">
@@ -1088,8 +1122,12 @@
           <t>ID / SIN</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr"/>
-      <c r="F13" s="7" t="n"/>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Academy SIN — FLAGGED</t>
+        </is>
+      </c>
+      <c r="F13" s="39" t="n"/>
       <c r="G13" s="3" t="n"/>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="n"/>
@@ -1178,13 +1216,6 @@
           <t>Sync rule: PDF is truth for stats, skills, chrome, dossier. This book is truth for €$, IP, heat, people, jobs. After a session: add a LEDGER row, then copy B11 / B12 / B15 onto PDF page 2.</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
       <c r="K18" s="3" t="n"/>
@@ -1196,13 +1227,6 @@
           <t>Photos: Insert → Pictures into the boxes on the right (booking + known photograph). Acrobat does the same on PDF page 0.</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="n"/>
@@ -1228,16 +1252,12 @@
           <t>BOOKING PHOTO</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
       <c r="D21" s="3" t="n"/>
       <c r="E21" s="12" t="inlineStr">
         <is>
           <t>KNOWN PHOTOGRAPH</t>
         </is>
       </c>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
       <c r="H21" s="3" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
@@ -1250,16 +1270,16 @@
           <t>Insert booking photo</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
+      <c r="B22" s="40" t="n"/>
+      <c r="C22" s="41" t="n"/>
       <c r="D22" s="3" t="n"/>
       <c r="E22" s="13" t="inlineStr">
         <is>
           <t>Insert street / known photo</t>
         </is>
       </c>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
+      <c r="F22" s="40" t="n"/>
+      <c r="G22" s="41" t="n"/>
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
@@ -1267,13 +1287,11 @@
       <c r="L22" s="3" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="3" t="n"/>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
+      <c r="A23" s="42" t="n"/>
+      <c r="C23" s="43" t="n"/>
       <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
+      <c r="E23" s="42" t="n"/>
+      <c r="G23" s="43" t="n"/>
       <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
@@ -1281,13 +1299,11 @@
       <c r="L23" s="3" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="3" t="n"/>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
+      <c r="A24" s="42" t="n"/>
+      <c r="C24" s="43" t="n"/>
       <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
+      <c r="E24" s="42" t="n"/>
+      <c r="G24" s="43" t="n"/>
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
@@ -1295,13 +1311,11 @@
       <c r="L24" s="3" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="3" t="n"/>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
+      <c r="A25" s="42" t="n"/>
+      <c r="C25" s="43" t="n"/>
       <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
+      <c r="E25" s="42" t="n"/>
+      <c r="G25" s="43" t="n"/>
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
@@ -1309,13 +1323,11 @@
       <c r="L25" s="3" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="3" t="n"/>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
+      <c r="A26" s="42" t="n"/>
+      <c r="C26" s="43" t="n"/>
       <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
+      <c r="E26" s="42" t="n"/>
+      <c r="G26" s="43" t="n"/>
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
@@ -1323,13 +1335,11 @@
       <c r="L26" s="3" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="3" t="n"/>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
+      <c r="A27" s="42" t="n"/>
+      <c r="C27" s="43" t="n"/>
       <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
+      <c r="E27" s="42" t="n"/>
+      <c r="G27" s="43" t="n"/>
       <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
@@ -1337,13 +1347,11 @@
       <c r="L27" s="3" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="3" t="n"/>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="n"/>
+      <c r="A28" s="42" t="n"/>
+      <c r="C28" s="43" t="n"/>
       <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
+      <c r="E28" s="42" t="n"/>
+      <c r="G28" s="43" t="n"/>
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
@@ -1351,13 +1359,11 @@
       <c r="L28" s="3" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="3" t="n"/>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
+      <c r="A29" s="42" t="n"/>
+      <c r="C29" s="43" t="n"/>
       <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n"/>
-      <c r="G29" s="3" t="n"/>
+      <c r="E29" s="42" t="n"/>
+      <c r="G29" s="43" t="n"/>
       <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
@@ -1365,13 +1371,13 @@
       <c r="L29" s="3" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="3" t="n"/>
-      <c r="B30" s="3" t="n"/>
-      <c r="C30" s="3" t="n"/>
+      <c r="A30" s="44" t="n"/>
+      <c r="B30" s="45" t="n"/>
+      <c r="C30" s="46" t="n"/>
       <c r="D30" s="3" t="n"/>
-      <c r="E30" s="3" t="n"/>
-      <c r="F30" s="3" t="n"/>
-      <c r="G30" s="3" t="n"/>
+      <c r="E30" s="44" t="n"/>
+      <c r="F30" s="45" t="n"/>
+      <c r="G30" s="46" t="n"/>
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
@@ -1493,7 +1499,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
@@ -1520,9 +1525,6 @@
           <t xml:space="preserve">  REF  ·  COMBAT  ·  CPR p.127–176, 186</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
       <c r="E1" s="3" t="n"/>
       <c r="F1" s="3" t="n"/>
       <c r="G1" s="3" t="n"/>
@@ -1552,9 +1554,6 @@
           <t>Turn = 1 Move Action + 1 other Action. Round ≈ 3 seconds. Initiative = REF + 1d10. Move = MOVE × 2 m (or MOVE squares, diagonals OK).</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
       <c r="E3" s="3" t="n"/>
       <c r="F3" s="3" t="n"/>
       <c r="G3" s="3" t="n"/>
@@ -1992,9 +1991,6 @@
           <t>WOUNDS  ·  ARMOR  ·  BRAWLING</t>
         </is>
       </c>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="n"/>
@@ -2010,9 +2006,9 @@
           <t>Seriously Wounded: HP ≤ ⌈HP max / 2⌉. −2 to all Actions. Death Save = BODY. Mortally Wounded: HP 0. At start of your Turn roll 1d10 ≤ BODY or die. Each time you take damage while Mortal: Critical Injury +1 Death Save Penalty.</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
+      <c r="B20" s="38" t="n"/>
+      <c r="C20" s="38" t="n"/>
+      <c r="D20" s="39" t="n"/>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="3" t="n"/>
@@ -2028,9 +2024,9 @@
           <t>Armor: if damage &gt; SP, HP loss = damage − SP, then ablate SP by 1 (unless the attack says otherwise). Melee weapons ignore half SP (round up). Brawling does NOT. Ablate Head and Body separately.</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
+      <c r="B21" s="38" t="n"/>
+      <c r="C21" s="38" t="n"/>
+      <c r="D21" s="39" t="n"/>
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n"/>
@@ -2046,9 +2042,9 @@
           <t>Brawling DMG by BODY: ≤4 → 1d6 · 5–6 (or ≤4 with Cyberarm) → 2d6 · 7–10 → 3d6 · 11+ → 4d6. Cyberarm brawl is at least 2d6.</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
+      <c r="B22" s="38" t="n"/>
+      <c r="C22" s="38" t="n"/>
+      <c r="D22" s="39" t="n"/>
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="n"/>
@@ -2064,9 +2060,9 @@
           <t>Facedown: both roll COOL + 1d10. Loser backs down or takes −2 on Checks against the winner until they beat them once. Cover: if they can see you, you are not in cover (bulletproof glass excepted).</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
+      <c r="B23" s="38" t="n"/>
+      <c r="C23" s="38" t="n"/>
+      <c r="D23" s="39" t="n"/>
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
       <c r="G23" s="3" t="n"/>
@@ -2082,9 +2078,9 @@
           <t>LUCK: spend 1:1 on a Check, resets each session. Extra Time: ×4 duration = +1 once. Complementary Skill: +1 once, no stack. Crit success: natural 10, add extra 1d10. Crit fail: natural 1, subtract extra 1d10.</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
+      <c r="B24" s="38" t="n"/>
+      <c r="C24" s="38" t="n"/>
+      <c r="D24" s="39" t="n"/>
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
       <c r="G24" s="3" t="n"/>
@@ -2314,14 +2310,6 @@
           <t xml:space="preserve">  REF  ·  RANGE TABLES  ·  CPR p.173–174</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
       <c r="J1" s="3" t="n"/>
       <c r="K1" s="3" t="n"/>
       <c r="L1" s="3" t="n"/>
@@ -2346,14 +2334,6 @@
           <t>Ranged: REF + weapon Skill + 1d10 vs DV by range (or vs DEX + Evasion + 1d10 if defender REF ≥ 8). Tie: defender wins. CPR p.173.</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="n"/>
@@ -2364,14 +2344,6 @@
           <t>SINGLE SHOT DV</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
       <c r="J4" s="3" t="n"/>
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="n"/>
@@ -2734,14 +2706,6 @@
           <t>AUTOFIRE DV   ·   costs 10 bullets  ·   Autofire Skill  ·   damage 2d6 × amount you beat DV, cap = weapon Autofire (SMG 3 / AR 4)  ·  no Aimed Shot</t>
         </is>
       </c>
-      <c r="B15" s="23" t="n"/>
-      <c r="C15" s="23" t="n"/>
-      <c r="D15" s="23" t="n"/>
-      <c r="E15" s="23" t="n"/>
-      <c r="F15" s="23" t="n"/>
-      <c r="G15" s="23" t="n"/>
-      <c r="H15" s="23" t="n"/>
-      <c r="I15" s="23" t="n"/>
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="3" t="n"/>
       <c r="L15" s="3" t="n"/>
@@ -2860,14 +2824,6 @@
           <t>Shotgun shell: 1 attack vs DV13; every target you can see in 6 m cone takes 3d6 (roll once). No Aimed Shot.</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
       <c r="K20" s="3" t="n"/>
       <c r="L20" s="3" t="n"/>
@@ -2878,14 +2834,6 @@
           <t>Suppressive Fire: Action + 10 bullets. Everyone on foot, out of cover, in LOS, ≤25 m: WILL + Concentration + 1d10 vs your REF + Autofire + 1d10 or they must Move into cover.</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
       <c r="K21" s="3" t="n"/>
       <c r="L21" s="3" t="n"/>
@@ -2896,14 +2844,6 @@
           <t>Thrown weapons: ROF 1, REF + Athletics vs thrown range DV. Melee thrown does not halve SP. Grenades deal explosive damage in 10×10 m.</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
       <c r="K22" s="3" t="n"/>
       <c r="L22" s="3" t="n"/>
@@ -2914,14 +2854,6 @@
           <t>Arrows: loading is part of the attack (no Reload Action). Basic arrows can be retrieved.</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
       <c r="K23" s="3" t="n"/>
       <c r="L23" s="3" t="n"/>
@@ -3155,9 +3087,6 @@
           <t xml:space="preserve">  REF  ·  DIFFICULTY  ·  IP  ·  PRICES  ·  CPR p.129–130, 385, 411</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
       <c r="E1" s="3" t="n"/>
       <c r="F1" s="3" t="n"/>
       <c r="G1" s="3" t="n"/>
@@ -3187,9 +3116,6 @@
           <t>STAT + Skill + 1d10 vs DV  (or vs defender STAT + Skill + 1d10). Tie: defender wins. No Skill: STAT + 1d10 only.</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
       <c r="E3" s="3" t="n"/>
       <c r="F3" s="3" t="n"/>
       <c r="G3" s="3" t="n"/>
@@ -3459,9 +3385,6 @@
           <t>IMPROVEMENT POINTS  (spend between sessions)</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
       <c r="G14" s="3" t="n"/>
@@ -3611,9 +3534,6 @@
           <t>PRICE CATEGORIES  ·  without a Fixer you buy up to Premium only</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="3" t="n"/>
@@ -3875,9 +3795,6 @@
           <t>Modifiers (subtract from your roll, they stack): night −1 · never done this −1 · complex −2 · no tools −2 · bad sleep −2 · extreme stress −2 · exhausted −4 · drunk/sedated −4 · secretly −4 · smoke/dark −4. Extra Time ×4 = +1. Complementary Skill = +1 once.</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n"/>
-      <c r="C31" s="3" t="n"/>
-      <c r="D31" s="3" t="n"/>
       <c r="E31" s="3" t="n"/>
       <c r="F31" s="3" t="n"/>
       <c r="G31" s="3" t="n"/>
@@ -3961,8 +3878,8 @@
   <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A3:D3"/>
     <mergeCell ref="A14:D14"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
@@ -4008,16 +3925,6 @@
           <t xml:space="preserve">  INCIDENT LOG   ·   OPERATOR LEDGER</t>
         </is>
       </c>
-      <c r="B1" s="9" t="n"/>
-      <c r="C1" s="9" t="n"/>
-      <c r="D1" s="9" t="n"/>
-      <c r="E1" s="9" t="n"/>
-      <c r="F1" s="9" t="n"/>
-      <c r="G1" s="9" t="n"/>
-      <c r="H1" s="9" t="n"/>
-      <c r="I1" s="9" t="n"/>
-      <c r="J1" s="9" t="n"/>
-      <c r="K1" s="9" t="n"/>
       <c r="L1" s="3" t="n"/>
     </row>
     <row r="2">
@@ -4093,17 +4000,55 @@
       <c r="L3" s="3" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="16" t="n"/>
-      <c r="G4" s="17" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>2076</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Floor 22, Megabuilding H5</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>NCPD / Glen warrant</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>H5 Valentinos; IA; scav BD</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>burned</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>NCPD personal · Glen aide · H5 Valentinos</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Warrant: take alive. Three down in the hall. Badge pulled. Radio in the drawer.</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Elena Ruiz (partner, on scene)</t>
+        </is>
+      </c>
       <c r="L4" s="3" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -4672,7 +4617,6 @@
           <t>Session €$ (this sheet)</t>
         </is>
       </c>
-      <c r="B45" s="3" t="n"/>
       <c r="C45" s="18">
         <f>SUM(F4:F43)</f>
         <v/>
@@ -4714,16 +4658,6 @@
           <t>In-world date, not real-world. Related persons should match CONTACTS handles. Heat = NCPD / corp / gang and a short note.</t>
         </is>
       </c>
-      <c r="B47" s="3" t="n"/>
-      <c r="C47" s="3" t="n"/>
-      <c r="D47" s="3" t="n"/>
-      <c r="E47" s="3" t="n"/>
-      <c r="F47" s="3" t="n"/>
-      <c r="G47" s="3" t="n"/>
-      <c r="H47" s="3" t="n"/>
-      <c r="I47" s="3" t="n"/>
-      <c r="J47" s="3" t="n"/>
-      <c r="K47" s="3" t="n"/>
       <c r="L47" s="3" t="n"/>
     </row>
   </sheetData>
@@ -4783,15 +4717,6 @@
           <t xml:space="preserve">  KNOWN ASSOCIATES   ·   CREW FILE</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
       <c r="K1" s="3" t="n"/>
       <c r="L1" s="3" t="n"/>
     </row>
@@ -4863,101 +4788,367 @@
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="n"/>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Elena Ruiz</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Elena Ruiz</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>NCPD beat</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>backup</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Ex-partner. Did not cover Floor 22. Did not sell him.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Backup call; precinct door</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>She owes nothing. He owes the report.</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Agent / HYW Vista locker</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Most poisonous phone on the list. Still picks up because Vista did not get better.</t>
+        </is>
+      </c>
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="n"/>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Dwyer</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Sgt. Frank Dwyer</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>NCPD desk, Heywood</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>backup</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Old desk. Thinks the city is already dead.</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Backup call; next-tier on a 6</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Dodge owes blood if heavies drop</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Heywood desk, not the radio net</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Named Backup Rank 4. A 6 on ETA is HIS people.</t>
+        </is>
+      </c>
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="3" t="n"/>
     </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Oz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Marcus Osorio</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>NCPD beat, Vista</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>backup</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Grew up on the same H5 stairs.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Backup call; street eyes on H5</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>even</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Vista beat / Mercado Sonora</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Rides while the bodies are “ours.”</t>
+        </is>
+      </c>
       <c r="K6" s="3" t="n"/>
       <c r="L6" s="3" t="n"/>
     </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Tran</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Kim Tran</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>NCPD beat</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>backup</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Other square. One call from duty.</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Backup call (once)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>She owes one call. Second camera flash and she dumps the number.</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Agent only</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Weakest link on the Rank 4 list. Do not burn her on a spectacle.</t>
+        </is>
+      </c>
       <c r="K7" s="3" t="n"/>
       <c r="L7" s="3" t="n"/>
     </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>El Sereno</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>(rumor — no booking)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Childhood stair-story, Megabuilding H5 after midnight.</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Do not hunt. Do not sell.</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>DO NOT TOUCH</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>H5 stairs after midnight</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Valued Person on the dossier. Myth Dodge made into a job. Not a choom.</t>
+        </is>
+      </c>
       <c r="K8" s="3" t="n"/>
       <c r="L8" s="3" t="n"/>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Los de H5</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>(crew, not a name)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Valentinos, H5 / Mercado / La Catrina</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>rival</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>The set that feeds the stack and moves bodies through La Catrina.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Heat; the notebook</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>war on the stack, not the whole family</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Mercado Sonora · La Catrina (Phalarope &amp; Plover)</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Floor 22 was theirs. Remaining names live in the jacket notebook.</t>
+        </is>
+      </c>
       <c r="K9" s="3" t="n"/>
       <c r="L9" s="3" t="n"/>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Glen aide</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>(no booking yet)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>municipal / Glen</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>rival</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Wanted the H5 mid-level alive. Got a process instead of a martyr.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Heat; why the badge came off</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>they wanted him living and discredited</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>The Glen / City Hall orbit</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Dirty politician lane. Do not make this a Valentinos war.</t>
+        </is>
+      </c>
       <c r="K10" s="3" t="n"/>
       <c r="L10" s="3" t="n"/>
     </row>
@@ -5163,15 +5354,6 @@
           <t>Other PCs at the table + recurring NPCs. Dossier page 0 only keeps name-lists; this sheet is the actual cards. Trust 1 = will burn you, 5 = choomba.</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="3" t="n"/>
-      <c r="J25" s="3" t="n"/>
       <c r="K25" s="3" t="n"/>
       <c r="L25" s="3" t="n"/>
     </row>
@@ -5380,11 +5562,6 @@
           <t xml:space="preserve">  NET   ·   INTERFACE / QUICKHACKS</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
       <c r="G1" s="3" t="n"/>
       <c r="H1" s="3" t="n"/>
       <c r="I1" s="3" t="n"/>
@@ -5412,8 +5589,12 @@
           <t>Cyberdeck</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="7" t="n"/>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C3" s="39" t="n"/>
       <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Interface Rank</t>
@@ -5444,7 +5625,11 @@
           <t>Self-ICE / Passwalls</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="F4" s="3" t="n"/>
       <c r="G4" s="3" t="n"/>
       <c r="H4" s="3" t="n"/>
@@ -5461,7 +5646,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="C5" s="3" t="n"/>
@@ -5470,7 +5655,11 @@
           <t>Ex-Disks</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="F5" s="3" t="n"/>
       <c r="G5" s="3" t="n"/>
       <c r="H5" s="3" t="n"/>
@@ -5499,11 +5688,6 @@
           <t>PROGRAMS  /  HARDWARE</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
@@ -5737,11 +5921,6 @@
           <t>QUICKHACKS  ·  CEMK 2070s  ·  Interface + 1d10 vs DV   (CPR p.197 / CEMK RB p.16–18, 39)</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
-      <c r="F22" s="9" t="n"/>
       <c r="G22" s="3" t="n"/>
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
@@ -5798,8 +5977,8 @@
           <t>MOVE −1 for 60s; 0 MOVE = no Move Action</t>
         </is>
       </c>
-      <c r="E24" s="26" t="n"/>
-      <c r="F24" s="26" t="n"/>
+      <c r="E24" s="38" t="n"/>
+      <c r="F24" s="39" t="n"/>
       <c r="G24" s="3" t="n"/>
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="n"/>
@@ -5826,8 +6005,8 @@
           <t>Damaged Ear crit (no bonus dmg) 60s</t>
         </is>
       </c>
-      <c r="E25" s="26" t="n"/>
-      <c r="F25" s="26" t="n"/>
+      <c r="E25" s="38" t="n"/>
+      <c r="F25" s="39" t="n"/>
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>
@@ -5854,8 +6033,8 @@
           <t>On fire: 4 HP at end of their Turn, bypass SP</t>
         </is>
       </c>
-      <c r="E26" s="26" t="n"/>
-      <c r="F26" s="26" t="n"/>
+      <c r="E26" s="38" t="n"/>
+      <c r="F26" s="39" t="n"/>
       <c r="G26" s="3" t="n"/>
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
@@ -5882,8 +6061,8 @@
           <t>GM picks 3 chrome pieces offline 60s</t>
         </is>
       </c>
-      <c r="E27" s="26" t="n"/>
-      <c r="F27" s="26" t="n"/>
+      <c r="E27" s="38" t="n"/>
+      <c r="F27" s="39" t="n"/>
       <c r="G27" s="3" t="n"/>
       <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="n"/>
@@ -5910,8 +6089,8 @@
           <t>You pick 1 chrome offline 60s (not Neuroport)</t>
         </is>
       </c>
-      <c r="E28" s="26" t="n"/>
-      <c r="F28" s="26" t="n"/>
+      <c r="E28" s="38" t="n"/>
+      <c r="F28" s="39" t="n"/>
       <c r="G28" s="3" t="n"/>
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n"/>
@@ -5938,8 +6117,8 @@
           <t>Force their next Move; only if unaware</t>
         </is>
       </c>
-      <c r="E29" s="26" t="n"/>
-      <c r="F29" s="26" t="n"/>
+      <c r="E29" s="38" t="n"/>
+      <c r="F29" s="39" t="n"/>
       <c r="G29" s="3" t="n"/>
       <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="n"/>
@@ -5966,8 +6145,8 @@
           <t>MOVE −1d6 for 60s</t>
         </is>
       </c>
-      <c r="E30" s="26" t="n"/>
-      <c r="F30" s="26" t="n"/>
+      <c r="E30" s="38" t="n"/>
+      <c r="F30" s="39" t="n"/>
       <c r="G30" s="3" t="n"/>
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n"/>
@@ -5994,8 +6173,8 @@
           <t>3d6 HP, bypass armor, no ablation</t>
         </is>
       </c>
-      <c r="E31" s="26" t="n"/>
-      <c r="F31" s="26" t="n"/>
+      <c r="E31" s="38" t="n"/>
+      <c r="F31" s="39" t="n"/>
       <c r="G31" s="3" t="n"/>
       <c r="H31" s="3" t="n"/>
       <c r="I31" s="3" t="n"/>
@@ -6022,8 +6201,8 @@
           <t>You spend their next Action + Move</t>
         </is>
       </c>
-      <c r="E32" s="26" t="n"/>
-      <c r="F32" s="26" t="n"/>
+      <c r="E32" s="38" t="n"/>
+      <c r="F32" s="39" t="n"/>
       <c r="G32" s="3" t="n"/>
       <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="n"/>
@@ -6050,8 +6229,8 @@
           <t>Eject 1 chipware into adjacent square</t>
         </is>
       </c>
-      <c r="E33" s="26" t="n"/>
-      <c r="F33" s="26" t="n"/>
+      <c r="E33" s="38" t="n"/>
+      <c r="F33" s="39" t="n"/>
       <c r="G33" s="3" t="n"/>
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="n"/>
@@ -6078,8 +6257,8 @@
           <t>Unconscious 60s or until damaged; Prone</t>
         </is>
       </c>
-      <c r="E34" s="26" t="n"/>
-      <c r="F34" s="26" t="n"/>
+      <c r="E34" s="38" t="n"/>
+      <c r="F34" s="39" t="n"/>
       <c r="G34" s="3" t="n"/>
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
@@ -6107,11 +6286,6 @@
           <t>Jack In: Interface + 1d10 vs target WILL + 1d10, 50 m, target must have a Neuroport. Failure still jacks in but they know. Eject: WILL + Concentration + 1d10 vs Interface + 1d10.</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="n"/>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
-      <c r="F36" s="3" t="n"/>
       <c r="G36" s="3" t="n"/>
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
@@ -6180,15 +6354,6 @@
           <t xml:space="preserve">  GARAGE   ·   MOTO / FAMILY MOTORPOOL</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
       <c r="K1" s="3" t="n"/>
       <c r="L1" s="3" t="n"/>
     </row>
@@ -6219,8 +6384,8 @@
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="7" t="n"/>
+      <c r="E3" s="38" t="n"/>
+      <c r="F3" s="39" t="n"/>
       <c r="G3" s="3" t="n"/>
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
@@ -6234,15 +6399,6 @@
           <t>Moto Rank adds to Drive/Pilot and Vehicle Tech checks. Only one Family Vehicle out at a time (all of them at Rank 10). CPR p.161–164.</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="n"/>
     </row>
@@ -6781,11 +6937,6 @@
           <t xml:space="preserve">  WORKSHOP   ·   MAKER</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
       <c r="G1" s="3" t="n"/>
       <c r="H1" s="3" t="n"/>
       <c r="I1" s="3" t="n"/>
@@ -6927,11 +7078,6 @@
           <t>Each Maker Rank: +1 to two different specialties. Field Expertise also jury-rigs as an Action. CPR p.147–149.</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
@@ -6959,11 +7105,6 @@
           <t>JOBS  ·  repairs, upgrades, inventions</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
@@ -7197,11 +7338,6 @@
           <t>Upgrade/Fabricate/Invent DV by price: Cheap 9 / 1h · Costly 13 / 6h · Premium 17 / 1d · Expensive 21 / 1w · V.Exp 24 / 2w · Luxury 29 / 1mo · Super Luxury 29 / 1mo per 10,000eb.</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>
@@ -7408,11 +7544,6 @@
           <t xml:space="preserve">  CLINIC   ·   MEDICINE</t>
         </is>
       </c>
-      <c r="B1" s="9" t="n"/>
-      <c r="C1" s="9" t="n"/>
-      <c r="D1" s="9" t="n"/>
-      <c r="E1" s="9" t="n"/>
-      <c r="F1" s="9" t="n"/>
       <c r="G1" s="3" t="n"/>
       <c r="H1" s="3" t="n"/>
       <c r="I1" s="3" t="n"/>
@@ -7518,11 +7649,6 @@
           <t>Each Medicine Rank: +1 to one specialty. Surgery Skill = 2 per point (max 10). Installation, harvesting, bodysculpt, therapy: CPR p.149, 226.</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
@@ -7550,11 +7676,6 @@
           <t>PATIENTS  /  THERAPY  /  PHARMA</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
@@ -8014,17 +8135,6 @@
           <t xml:space="preserve">  TEAM   ·   EXEC TEAMWORK</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n"/>
@@ -8053,8 +8163,8 @@
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="7" t="n"/>
+      <c r="E3" s="38" t="n"/>
+      <c r="F3" s="39" t="n"/>
       <c r="G3" s="3" t="n"/>
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
@@ -8068,17 +8178,6 @@
           <t>Exec team members are mechanical NPCs, not just CONTACTS. Use cover job / true job. CPR p.153–157 for who you get at each Rank.</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
@@ -8623,11 +8722,6 @@
           <t xml:space="preserve">  WISHLIST   ·   NIGHT MARKET</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
       <c r="G1" s="3" t="n"/>
       <c r="H1" s="3" t="n"/>
       <c r="I1" s="3" t="n"/>
@@ -8688,12 +8782,34 @@
       <c r="L3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr"/>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="16" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Neuroport</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>cyberware</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Very Expensive</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Hospital / ripper</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>House rule: not free. HL 7 (2d6). Required for other chrome.</t>
+        </is>
+      </c>
       <c r="G4" s="3" t="n"/>
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="n"/>
@@ -8702,12 +8818,34 @@
       <c r="L4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr"/>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="16" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Self-ICE</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>cyberware</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Expensive</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>500</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Needs Neuroport. Quickhack Passwall.</t>
+        </is>
+      </c>
       <c r="G5" s="3" t="n"/>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
@@ -8716,12 +8854,34 @@
       <c r="L5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="16" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NCPD Crime Database</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>gear / Agent</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Expensive</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>500</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>stolen login / GM</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Skiptrace sugar. Badge is pulled — access is a plot.</t>
+        </is>
+      </c>
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
@@ -8730,12 +8890,34 @@
       <c r="L6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr"/>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="16" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Light Armorjack (Head)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Night Market</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>If the mirrorshades stop being enough.</t>
+        </is>
+      </c>
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
@@ -8744,12 +8926,34 @@
       <c r="L7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr"/>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="16" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr"/>
-      <c r="F8" s="5" t="inlineStr"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Basic Heavy Pistol ammo x50</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>ammo</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Cheap</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Unity food.</t>
+        </is>
+      </c>
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
@@ -8758,12 +8962,34 @@
       <c r="L8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr"/>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="16" t="inlineStr"/>
-      <c r="E9" s="5" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Explosive Slug x10</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>ammo</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Fixer</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Satara barrel B.</t>
+        </is>
+      </c>
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
@@ -8987,11 +9213,6 @@
           <t>Price categories (CPR p.385): Cheap 10 · Everyday 20 · Costly 50 · Premium 100 · Expensive 500 · Very Expensive 1,000 · Luxury 5,000 · Super Luxury 10,000+.</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>

</xml_diff>

<commit_message>
Fill Night Shift Street File with DODGE, keep template chrome
Restore the Night Shift PDF/xlsx shells and write Rafael "DODGE" Mora on top (Lawman 4, H5). Portraits stay empty. xlsx keeps NCPD/operator marks; META, Floor 22 ledger, named Backup contacts.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sheets/Street-File.xlsx
+++ b/sheets/Street-File.xlsx
@@ -457,6 +457,61 @@
 </comments>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LEDGER" displayName="LEDGER" ref="A3:K43" headerRowCount="1">
   <autoFilter ref="A3:K43"/>
@@ -1499,6 +1554,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Embed DODGE booking and known photos in Street File
Paste the two uploads/ portraits into PDF page 1 photo frames and META photo boxes on the xlsx, keeping Night Shift chrome.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sheets/Street-File.xlsx
+++ b/sheets/Street-File.xlsx
@@ -509,6 +509,56 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2000250" cy="2800350"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Booking" descr="Booking photo"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2000250" cy="2800350"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Known" descr="Known photograph"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 

</xml_diff>